<commit_message>
Record the Playwright run results in the QA workbook
54 of 263 cases now carry an observed result, up from 47. The 25 new
ones come from the black-box Playwright suite in D:\flexicaai-qa and are
evidenced on a new "Playwright Run" sheet.

The suite lives outside this repo deliberately: it imports no
application source, so it can disagree with the code rather than agree
with its bugs, and QA can own it on its own cadence. No Playwright
dependency is added here.

Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/qa/Clinic_Management_Complete_QA_Test_Cases.xlsx
+++ b/docs/qa/Clinic_Management_Complete_QA_Test_Cases.xlsx
@@ -10,13 +10,14 @@
     <sheet sheetId="4" name="Feature Coverage" state="visible" r:id="rId7"/>
     <sheet sheetId="5" name="Read Me First" state="visible" r:id="rId8"/>
     <sheet sheetId="6" name="Automated Run" state="visible" r:id="rId9"/>
+    <sheet sheetId="7" name="Playwright Run" state="visible" r:id="rId10"/>
   </sheets>
   <calcPr calcId="171027"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2924" uniqueCount="1742">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3005" uniqueCount="1770">
   <si>
     <t>Test Case ID</t>
   </si>
@@ -6448,12 +6449,96 @@
   <si>
     <t>47 of 263 cases were executed automatically against the running application on 2026-10-05 and carry an observed result. The remaining 216 are left BLANK deliberately: they need a human to judge the outcome, test data this run did not create, or a credential this environment does not have. A result nobody observed would be worse than an empty cell.</t>
   </si>
+  <si>
+    <t>What the automated run did</t>
+  </si>
+  <si>
+    <t>Automated (Playwright): all four clinic roles sign in and land in the workspace</t>
+  </si>
+  <si>
+    <t>Automated (Playwright): unknown username is refused without revealing it does not exist</t>
+  </si>
+  <si>
+    <t>Automated (Playwright): a wrong password gives the identical message</t>
+  </si>
+  <si>
+    <t>Automated (Playwright): empty fields are blocked before any request</t>
+  </si>
+  <si>
+    <t>Automated (Playwright): a suspended account is refused after the password is checked</t>
+  </si>
+  <si>
+    <t>Automated (Playwright): signing out ends the session and protected pages stay unreachable</t>
+  </si>
+  <si>
+    <t>Automated (Playwright): anonymous visits to protected pages redirect to login</t>
+  </si>
+  <si>
+    <t>Automated (Playwright): a deep link is not restored after signing in</t>
+  </si>
+  <si>
+    <t>Automated (Playwright): doctor sees clinical items and no money or staff items</t>
+  </si>
+  <si>
+    <t>Automated (Playwright): receptionist sees the money screens but not the scribe</t>
+  </si>
+  <si>
+    <t>Automated (Playwright): manager sees neither staff nor expenses</t>
+  </si>
+  <si>
+    <t>Automated (Playwright): doctor cannot reach staff management by URL</t>
+  </si>
+  <si>
+    <t>Automated (Playwright): receptionist is bounced from every restricted screen</t>
+  </si>
+  <si>
+    <t>Automated (Playwright): manager cannot reach staff, expenses or profit and loss</t>
+  </si>
+  <si>
+    <t>Automated (Playwright): a clinic admin cannot enter the company panel</t>
+  </si>
+  <si>
+    <t>Automated (Playwright): receptionist cannot reach the voice scribe</t>
+  </si>
+  <si>
+    <t>Automated (Playwright): manager opens the scribe page but is offered no recorder</t>
+  </si>
+  <si>
+    <t>Automated (Playwright): create a patient with every field completed</t>
+  </si>
+  <si>
+    <t>Automated (Playwright): create a patient with only the two mandatory fields</t>
+  </si>
+  <si>
+    <t>Automated (Playwright): a patient cannot be saved without a name</t>
+  </si>
+  <si>
+    <t>Automated (Playwright): a patient cannot be saved without a phone number</t>
+  </si>
+  <si>
+    <t>Automated (Playwright): search finds a patient by name and filters the rest out</t>
+  </si>
+  <si>
+    <t>Automated (Playwright): a search with no matches shows an empty state rather than an error</t>
+  </si>
+  <si>
+    <t>Automated (Playwright): another clinic's patient cannot be opened by id</t>
+  </si>
+  <si>
+    <t>Automated (Playwright): doctor can read patients but is offered no create control</t>
+  </si>
+  <si>
+    <t>SOURCE</t>
+  </si>
+  <si>
+    <t>Produced by the Playwright suite in D:\flexicaai-qa on 2026-10-05 20:47. Full evidence — traces, screenshots and video for any failure — is in reports/html; open it with "npm run report". Rows with no result are NOT failures: they need a human, and are deliberately left blank.</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="12" x14ac:knownFonts="1">
+  <fonts count="13" x14ac:knownFonts="1">
     <font>
       <color theme="1"/>
       <family val="2"/>
@@ -6497,11 +6582,15 @@
       <sz val="12"/>
     </font>
     <font>
-      <sz val="10.5"/>
+      <b/>
+      <color rgb="FF1B6B38"/>
     </font>
     <font>
-      <b/>
-      <color rgb="FF1B6B38"/>
+      <i/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <sz val="10.5"/>
     </font>
     <font>
       <i/>
@@ -6557,7 +6646,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="19">
+  <cellXfs count="20">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
@@ -6609,6 +6698,9 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -8367,7 +8459,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="55" spans="1:8" s="5" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A55" s="3" t="s">
         <v>303</v>
       </c>
@@ -8390,10 +8482,10 @@
         <v>308</v>
       </c>
       <c r="H55" s="4" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="56" spans="1:8" s="6" customFormat="1" x14ac:dyDescent="0.25">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="56" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A56" s="3" t="s">
         <v>309</v>
       </c>
@@ -8416,10 +8508,10 @@
         <v>312</v>
       </c>
       <c r="H56" s="4" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="57" spans="1:8" s="5" customFormat="1" x14ac:dyDescent="0.25">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="57" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A57" s="3" t="s">
         <v>313</v>
       </c>
@@ -8442,10 +8534,10 @@
         <v>318</v>
       </c>
       <c r="H57" s="4" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="58" spans="1:8" s="6" customFormat="1" x14ac:dyDescent="0.25">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="58" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A58" s="3" t="s">
         <v>319</v>
       </c>
@@ -8468,7 +8560,7 @@
         <v>322</v>
       </c>
       <c r="H58" s="4" t="s">
-        <v>41</v>
+        <v>15</v>
       </c>
     </row>
     <row r="59" spans="1:8" s="5" customFormat="1" x14ac:dyDescent="0.25">
@@ -8601,7 +8693,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="64" spans="1:8" s="6" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A64" s="3" t="s">
         <v>348</v>
       </c>
@@ -8624,10 +8716,10 @@
         <v>353</v>
       </c>
       <c r="H64" s="4" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="65" spans="1:8" s="5" customFormat="1" x14ac:dyDescent="0.25">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="65" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A65" s="3" t="s">
         <v>354</v>
       </c>
@@ -8650,7 +8742,7 @@
         <v>358</v>
       </c>
       <c r="H65" s="4" t="s">
-        <v>41</v>
+        <v>15</v>
       </c>
     </row>
     <row r="66" spans="1:8" s="6" customFormat="1" x14ac:dyDescent="0.25">
@@ -8731,7 +8823,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="69" spans="1:8" s="5" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A69" s="3" t="s">
         <v>375</v>
       </c>
@@ -8754,7 +8846,7 @@
         <v>380</v>
       </c>
       <c r="H69" s="4" t="s">
-        <v>41</v>
+        <v>15</v>
       </c>
     </row>
     <row r="70" spans="1:8" s="6" customFormat="1" x14ac:dyDescent="0.25">
@@ -17032,532 +17124,845 @@
         <v>1692</v>
       </c>
     </row>
-    <row r="2" spans="1:3" s="16" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="16" t="s">
+    <row r="2" spans="1:3" s="13" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A2" s="13" t="s">
         <v>8</v>
       </c>
-      <c r="B2" s="17" t="s">
+      <c r="B2" s="16" t="s">
         <v>15</v>
       </c>
-      <c r="C2" s="16" t="s">
+      <c r="C2" s="13" t="s">
         <v>1693</v>
       </c>
     </row>
-    <row r="3" spans="1:3" s="16" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="16" t="s">
+    <row r="3" spans="1:3" s="13" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A3" s="13" t="s">
         <v>16</v>
       </c>
-      <c r="B3" s="17" t="s">
+      <c r="B3" s="16" t="s">
         <v>15</v>
       </c>
-      <c r="C3" s="16" t="s">
+      <c r="C3" s="13" t="s">
         <v>1694</v>
       </c>
     </row>
-    <row r="4" spans="1:3" s="16" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="16" t="s">
+    <row r="4" spans="1:3" s="13" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A4" s="13" t="s">
         <v>21</v>
       </c>
-      <c r="B4" s="17" t="s">
+      <c r="B4" s="16" t="s">
         <v>15</v>
       </c>
-      <c r="C4" s="16" t="s">
+      <c r="C4" s="13" t="s">
         <v>1695</v>
       </c>
     </row>
-    <row r="5" spans="1:3" s="16" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="16" t="s">
+    <row r="5" spans="1:3" s="13" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A5" s="13" t="s">
         <v>26</v>
       </c>
-      <c r="B5" s="17" t="s">
+      <c r="B5" s="16" t="s">
         <v>15</v>
       </c>
-      <c r="C5" s="16" t="s">
+      <c r="C5" s="13" t="s">
         <v>1696</v>
       </c>
     </row>
-    <row r="6" spans="1:3" s="16" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="16" t="s">
+    <row r="6" spans="1:3" s="13" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A6" s="13" t="s">
         <v>31</v>
       </c>
-      <c r="B6" s="17" t="s">
+      <c r="B6" s="16" t="s">
         <v>15</v>
       </c>
-      <c r="C6" s="16" t="s">
+      <c r="C6" s="13" t="s">
         <v>1697</v>
       </c>
     </row>
-    <row r="7" spans="1:3" s="16" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="16" t="s">
+    <row r="7" spans="1:3" s="13" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A7" s="13" t="s">
         <v>42</v>
       </c>
-      <c r="B7" s="17" t="s">
+      <c r="B7" s="16" t="s">
         <v>15</v>
       </c>
-      <c r="C7" s="16" t="s">
+      <c r="C7" s="13" t="s">
         <v>1698</v>
       </c>
     </row>
-    <row r="8" spans="1:3" s="16" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="16" t="s">
+    <row r="8" spans="1:3" s="13" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A8" s="13" t="s">
         <v>159</v>
       </c>
-      <c r="B8" s="17" t="s">
+      <c r="B8" s="16" t="s">
         <v>15</v>
       </c>
-      <c r="C8" s="16" t="s">
+      <c r="C8" s="13" t="s">
         <v>1699</v>
       </c>
     </row>
-    <row r="9" spans="1:3" s="16" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="16" t="s">
+    <row r="9" spans="1:3" s="13" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A9" s="13" t="s">
         <v>165</v>
       </c>
-      <c r="B9" s="17" t="s">
+      <c r="B9" s="16" t="s">
         <v>15</v>
       </c>
-      <c r="C9" s="16" t="s">
+      <c r="C9" s="13" t="s">
         <v>1700</v>
       </c>
     </row>
-    <row r="10" spans="1:3" s="16" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="16" t="s">
+    <row r="10" spans="1:3" s="13" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A10" s="13" t="s">
         <v>138</v>
       </c>
-      <c r="B10" s="17" t="s">
+      <c r="B10" s="16" t="s">
         <v>15</v>
       </c>
-      <c r="C10" s="16" t="s">
+      <c r="C10" s="13" t="s">
         <v>1701</v>
       </c>
     </row>
-    <row r="11" spans="1:3" s="16" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="16" t="s">
+    <row r="11" spans="1:3" s="13" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A11" s="13" t="s">
         <v>176</v>
       </c>
-      <c r="B11" s="17" t="s">
+      <c r="B11" s="16" t="s">
         <v>15</v>
       </c>
-      <c r="C11" s="16" t="s">
+      <c r="C11" s="13" t="s">
         <v>1702</v>
       </c>
     </row>
-    <row r="12" spans="1:3" s="16" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="16" t="s">
+    <row r="12" spans="1:3" s="13" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A12" s="13" t="s">
         <v>183</v>
       </c>
-      <c r="B12" s="17" t="s">
+      <c r="B12" s="16" t="s">
         <v>15</v>
       </c>
-      <c r="C12" s="16" t="s">
+      <c r="C12" s="13" t="s">
         <v>1703</v>
       </c>
     </row>
-    <row r="13" spans="1:3" s="16" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="16" t="s">
+    <row r="13" spans="1:3" s="13" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A13" s="13" t="s">
         <v>189</v>
       </c>
-      <c r="B13" s="17" t="s">
+      <c r="B13" s="16" t="s">
         <v>15</v>
       </c>
-      <c r="C13" s="16" t="s">
+      <c r="C13" s="13" t="s">
         <v>1704</v>
       </c>
     </row>
-    <row r="14" spans="1:3" s="16" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="16" t="s">
+    <row r="14" spans="1:3" s="13" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A14" s="13" t="s">
         <v>195</v>
       </c>
-      <c r="B14" s="17" t="s">
+      <c r="B14" s="16" t="s">
         <v>15</v>
       </c>
-      <c r="C14" s="16" t="s">
+      <c r="C14" s="13" t="s">
         <v>1705</v>
       </c>
     </row>
-    <row r="15" spans="1:3" s="16" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="16" t="s">
+    <row r="15" spans="1:3" s="13" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A15" s="13" t="s">
         <v>201</v>
       </c>
-      <c r="B15" s="17" t="s">
+      <c r="B15" s="16" t="s">
         <v>15</v>
       </c>
-      <c r="C15" s="16" t="s">
+      <c r="C15" s="13" t="s">
         <v>1706</v>
       </c>
     </row>
-    <row r="16" spans="1:3" s="16" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="16" t="s">
+    <row r="16" spans="1:3" s="13" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A16" s="13" t="s">
         <v>206</v>
       </c>
-      <c r="B16" s="17" t="s">
+      <c r="B16" s="16" t="s">
         <v>15</v>
       </c>
-      <c r="C16" s="16" t="s">
+      <c r="C16" s="13" t="s">
         <v>1707</v>
       </c>
     </row>
-    <row r="17" spans="1:3" s="16" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A17" s="16" t="s">
+    <row r="17" spans="1:3" s="13" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A17" s="13" t="s">
         <v>211</v>
       </c>
-      <c r="B17" s="17" t="s">
+      <c r="B17" s="16" t="s">
         <v>15</v>
       </c>
-      <c r="C17" s="16" t="s">
+      <c r="C17" s="13" t="s">
         <v>1708</v>
       </c>
     </row>
-    <row r="18" spans="1:3" s="16" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A18" s="16" t="s">
+    <row r="18" spans="1:3" s="13" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A18" s="13" t="s">
         <v>558</v>
       </c>
-      <c r="B18" s="17" t="s">
+      <c r="B18" s="16" t="s">
         <v>15</v>
       </c>
-      <c r="C18" s="16" t="s">
+      <c r="C18" s="13" t="s">
         <v>1709</v>
       </c>
     </row>
-    <row r="19" spans="1:3" s="16" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A19" s="16" t="s">
+    <row r="19" spans="1:3" s="13" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A19" s="13" t="s">
         <v>563</v>
       </c>
-      <c r="B19" s="17" t="s">
+      <c r="B19" s="16" t="s">
         <v>15</v>
       </c>
-      <c r="C19" s="16" t="s">
+      <c r="C19" s="13" t="s">
         <v>1710</v>
       </c>
     </row>
-    <row r="20" spans="1:3" s="16" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A20" s="16" t="s">
+    <row r="20" spans="1:3" s="13" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A20" s="13" t="s">
         <v>229</v>
       </c>
-      <c r="B20" s="17" t="s">
+      <c r="B20" s="16" t="s">
         <v>15</v>
       </c>
-      <c r="C20" s="16" t="s">
+      <c r="C20" s="13" t="s">
         <v>1711</v>
       </c>
     </row>
-    <row r="21" spans="1:3" s="16" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A21" s="16" t="s">
+    <row r="21" spans="1:3" s="13" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A21" s="13" t="s">
         <v>222</v>
       </c>
-      <c r="B21" s="17" t="s">
+      <c r="B21" s="16" t="s">
         <v>15</v>
       </c>
-      <c r="C21" s="16" t="s">
+      <c r="C21" s="13" t="s">
         <v>1712</v>
       </c>
     </row>
-    <row r="22" spans="1:3" s="16" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A22" s="16" t="s">
+    <row r="22" spans="1:3" s="13" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A22" s="13" t="s">
         <v>398</v>
       </c>
-      <c r="B22" s="17" t="s">
+      <c r="B22" s="16" t="s">
         <v>15</v>
       </c>
-      <c r="C22" s="16" t="s">
+      <c r="C22" s="13" t="s">
         <v>1713</v>
       </c>
     </row>
-    <row r="23" spans="1:3" s="16" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A23" s="16" t="s">
+    <row r="23" spans="1:3" s="13" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A23" s="13" t="s">
         <v>387</v>
       </c>
-      <c r="B23" s="17" t="s">
+      <c r="B23" s="16" t="s">
         <v>15</v>
       </c>
-      <c r="C23" s="16" t="s">
+      <c r="C23" s="13" t="s">
         <v>1714</v>
       </c>
     </row>
-    <row r="24" spans="1:3" s="16" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A24" s="16" t="s">
+    <row r="24" spans="1:3" s="13" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A24" s="13" t="s">
         <v>1224</v>
       </c>
-      <c r="B24" s="17" t="s">
+      <c r="B24" s="16" t="s">
         <v>15</v>
       </c>
-      <c r="C24" s="16" t="s">
+      <c r="C24" s="13" t="s">
         <v>1715</v>
       </c>
     </row>
-    <row r="25" spans="1:3" s="16" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A25" s="16" t="s">
+    <row r="25" spans="1:3" s="13" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A25" s="13" t="s">
         <v>490</v>
       </c>
-      <c r="B25" s="17" t="s">
+      <c r="B25" s="16" t="s">
         <v>15</v>
       </c>
-      <c r="C25" s="16" t="s">
+      <c r="C25" s="13" t="s">
         <v>1716</v>
       </c>
     </row>
-    <row r="26" spans="1:3" s="16" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A26" s="16" t="s">
+    <row r="26" spans="1:3" s="13" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A26" s="13" t="s">
         <v>496</v>
       </c>
-      <c r="B26" s="17" t="s">
+      <c r="B26" s="16" t="s">
         <v>15</v>
       </c>
-      <c r="C26" s="16" t="s">
+      <c r="C26" s="13" t="s">
         <v>1717</v>
       </c>
     </row>
-    <row r="27" spans="1:3" s="16" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A27" s="16" t="s">
+    <row r="27" spans="1:3" s="13" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A27" s="13" t="s">
         <v>502</v>
       </c>
-      <c r="B27" s="17" t="s">
+      <c r="B27" s="16" t="s">
         <v>15</v>
       </c>
-      <c r="C27" s="16" t="s">
+      <c r="C27" s="13" t="s">
         <v>1718</v>
       </c>
     </row>
-    <row r="28" spans="1:3" s="16" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A28" s="16" t="s">
+    <row r="28" spans="1:3" s="13" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A28" s="13" t="s">
         <v>919</v>
       </c>
-      <c r="B28" s="17" t="s">
+      <c r="B28" s="16" t="s">
         <v>15</v>
       </c>
-      <c r="C28" s="16" t="s">
+      <c r="C28" s="13" t="s">
         <v>1719</v>
       </c>
     </row>
-    <row r="29" spans="1:3" s="16" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A29" s="16" t="s">
+    <row r="29" spans="1:3" s="13" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A29" s="13" t="s">
         <v>925</v>
       </c>
-      <c r="B29" s="17" t="s">
+      <c r="B29" s="16" t="s">
         <v>15</v>
       </c>
-      <c r="C29" s="16" t="s">
+      <c r="C29" s="13" t="s">
         <v>1720</v>
       </c>
     </row>
-    <row r="30" spans="1:3" s="16" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A30" s="16" t="s">
+    <row r="30" spans="1:3" s="13" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A30" s="13" t="s">
         <v>790</v>
       </c>
-      <c r="B30" s="17" t="s">
+      <c r="B30" s="16" t="s">
         <v>15</v>
       </c>
-      <c r="C30" s="16" t="s">
+      <c r="C30" s="13" t="s">
         <v>1721</v>
       </c>
     </row>
-    <row r="31" spans="1:3" s="16" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A31" s="16" t="s">
+    <row r="31" spans="1:3" s="13" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A31" s="13" t="s">
         <v>784</v>
       </c>
-      <c r="B31" s="17" t="s">
+      <c r="B31" s="16" t="s">
         <v>15</v>
       </c>
-      <c r="C31" s="16" t="s">
+      <c r="C31" s="13" t="s">
         <v>1722</v>
       </c>
     </row>
-    <row r="32" spans="1:3" s="16" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A32" s="16" t="s">
+    <row r="32" spans="1:3" s="13" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A32" s="13" t="s">
         <v>795</v>
       </c>
-      <c r="B32" s="17" t="s">
+      <c r="B32" s="16" t="s">
         <v>15</v>
       </c>
-      <c r="C32" s="16" t="s">
+      <c r="C32" s="13" t="s">
         <v>1723</v>
       </c>
     </row>
-    <row r="33" spans="1:3" s="16" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A33" s="16" t="s">
+    <row r="33" spans="1:3" s="13" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A33" s="13" t="s">
         <v>801</v>
       </c>
-      <c r="B33" s="17" t="s">
+      <c r="B33" s="16" t="s">
         <v>15</v>
       </c>
-      <c r="C33" s="16" t="s">
+      <c r="C33" s="13" t="s">
         <v>1724</v>
       </c>
     </row>
-    <row r="34" spans="1:3" s="16" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A34" s="16" t="s">
+    <row r="34" spans="1:3" s="13" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A34" s="13" t="s">
         <v>818</v>
       </c>
-      <c r="B34" s="17" t="s">
+      <c r="B34" s="16" t="s">
         <v>15</v>
       </c>
-      <c r="C34" s="16" t="s">
+      <c r="C34" s="13" t="s">
         <v>1725</v>
       </c>
     </row>
-    <row r="35" spans="1:3" s="16" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A35" s="16" t="s">
+    <row r="35" spans="1:3" s="13" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A35" s="13" t="s">
         <v>824</v>
       </c>
-      <c r="B35" s="17" t="s">
+      <c r="B35" s="16" t="s">
         <v>15</v>
       </c>
-      <c r="C35" s="16" t="s">
+      <c r="C35" s="13" t="s">
         <v>1726</v>
       </c>
     </row>
-    <row r="36" spans="1:3" s="16" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A36" s="16" t="s">
+    <row r="36" spans="1:3" s="13" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A36" s="13" t="s">
         <v>853</v>
       </c>
-      <c r="B36" s="17" t="s">
+      <c r="B36" s="16" t="s">
         <v>15</v>
       </c>
-      <c r="C36" s="16" t="s">
+      <c r="C36" s="13" t="s">
         <v>1727</v>
       </c>
     </row>
-    <row r="37" spans="1:3" s="16" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A37" s="16" t="s">
+    <row r="37" spans="1:3" s="13" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A37" s="13" t="s">
         <v>1072</v>
       </c>
-      <c r="B37" s="17" t="s">
+      <c r="B37" s="16" t="s">
         <v>15</v>
       </c>
-      <c r="C37" s="16" t="s">
+      <c r="C37" s="13" t="s">
         <v>1728</v>
       </c>
     </row>
-    <row r="38" spans="1:3" s="16" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A38" s="16" t="s">
+    <row r="38" spans="1:3" s="13" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A38" s="13" t="s">
         <v>1130</v>
       </c>
-      <c r="B38" s="17" t="s">
+      <c r="B38" s="16" t="s">
         <v>15</v>
       </c>
-      <c r="C38" s="16" t="s">
+      <c r="C38" s="13" t="s">
         <v>1729</v>
       </c>
     </row>
-    <row r="39" spans="1:3" s="16" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A39" s="16" t="s">
+    <row r="39" spans="1:3" s="13" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A39" s="13" t="s">
         <v>1136</v>
       </c>
-      <c r="B39" s="17" t="s">
+      <c r="B39" s="16" t="s">
         <v>15</v>
       </c>
-      <c r="C39" s="16" t="s">
+      <c r="C39" s="13" t="s">
         <v>1730</v>
       </c>
     </row>
-    <row r="40" spans="1:3" s="16" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A40" s="16" t="s">
+    <row r="40" spans="1:3" s="13" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A40" s="13" t="s">
         <v>1141</v>
       </c>
-      <c r="B40" s="17" t="s">
+      <c r="B40" s="16" t="s">
         <v>15</v>
       </c>
-      <c r="C40" s="16" t="s">
+      <c r="C40" s="13" t="s">
         <v>1731</v>
       </c>
     </row>
-    <row r="41" spans="1:3" s="16" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A41" s="16" t="s">
+    <row r="41" spans="1:3" s="13" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A41" s="13" t="s">
         <v>842</v>
       </c>
-      <c r="B41" s="17" t="s">
+      <c r="B41" s="16" t="s">
         <v>15</v>
       </c>
-      <c r="C41" s="16" t="s">
+      <c r="C41" s="13" t="s">
         <v>1732</v>
       </c>
     </row>
-    <row r="42" spans="1:3" s="16" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A42" s="16" t="s">
+    <row r="42" spans="1:3" s="13" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A42" s="13" t="s">
         <v>836</v>
       </c>
-      <c r="B42" s="17" t="s">
+      <c r="B42" s="16" t="s">
         <v>15</v>
       </c>
-      <c r="C42" s="16" t="s">
+      <c r="C42" s="13" t="s">
         <v>1733</v>
       </c>
     </row>
-    <row r="43" spans="1:3" s="16" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A43" s="16" t="s">
+    <row r="43" spans="1:3" s="13" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A43" s="13" t="s">
         <v>847</v>
       </c>
-      <c r="B43" s="17" t="s">
+      <c r="B43" s="16" t="s">
         <v>15</v>
       </c>
-      <c r="C43" s="16" t="s">
+      <c r="C43" s="13" t="s">
         <v>1734</v>
       </c>
     </row>
-    <row r="44" spans="1:3" s="16" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A44" s="16" t="s">
+    <row r="44" spans="1:3" s="13" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A44" s="13" t="s">
         <v>930</v>
       </c>
-      <c r="B44" s="17" t="s">
+      <c r="B44" s="16" t="s">
         <v>15</v>
       </c>
-      <c r="C44" s="16" t="s">
+      <c r="C44" s="13" t="s">
         <v>1735</v>
       </c>
     </row>
-    <row r="45" spans="1:3" s="16" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A45" s="16" t="s">
+    <row r="45" spans="1:3" s="13" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A45" s="13" t="s">
         <v>508</v>
       </c>
-      <c r="B45" s="17" t="s">
+      <c r="B45" s="16" t="s">
         <v>15</v>
       </c>
-      <c r="C45" s="16" t="s">
+      <c r="C45" s="13" t="s">
         <v>1736</v>
       </c>
     </row>
-    <row r="46" spans="1:3" s="16" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A46" s="16" t="s">
+    <row r="46" spans="1:3" s="13" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A46" s="13" t="s">
         <v>1259</v>
       </c>
-      <c r="B46" s="17" t="s">
+      <c r="B46" s="16" t="s">
         <v>15</v>
       </c>
-      <c r="C46" s="16" t="s">
+      <c r="C46" s="13" t="s">
         <v>1737</v>
       </c>
     </row>
-    <row r="47" spans="1:3" s="16" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A47" s="16" t="s">
+    <row r="47" spans="1:3" s="13" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A47" s="13" t="s">
         <v>542</v>
       </c>
-      <c r="B47" s="17" t="s">
+      <c r="B47" s="16" t="s">
         <v>15</v>
       </c>
-      <c r="C47" s="16" t="s">
+      <c r="C47" s="13" t="s">
         <v>1738</v>
       </c>
     </row>
-    <row r="48" spans="1:3" s="16" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A48" s="16" t="s">
+    <row r="48" spans="1:3" s="13" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A48" s="13" t="s">
         <v>547</v>
       </c>
-      <c r="B48" s="17" t="s">
+      <c r="B48" s="16" t="s">
         <v>15</v>
       </c>
-      <c r="C48" s="16" t="s">
+      <c r="C48" s="13" t="s">
         <v>1739</v>
       </c>
     </row>
-    <row r="50" spans="1:3" s="18" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A50" s="18" t="s">
+    <row r="50" spans="1:3" s="17" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A50" s="17" t="s">
         <v>1740</v>
       </c>
-      <c r="B50" s="18" t="s">
-        <v>41</v>
-      </c>
-      <c r="C50" s="18" t="s">
+      <c r="B50" s="17" t="s">
+        <v>41</v>
+      </c>
+      <c r="C50" s="17" t="s">
         <v>1741</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:C28"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <cols>
+    <col min="1" max="1" width="18" customWidth="1"/>
+    <col min="2" max="2" width="10" customWidth="1"/>
+    <col min="3" max="3" width="120" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" s="10" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="10" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="10" t="s">
+        <v>1691</v>
+      </c>
+      <c r="C1" s="10" t="s">
+        <v>1742</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" s="18" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A2" s="18" t="s">
+        <v>8</v>
+      </c>
+      <c r="B2" s="16" t="s">
+        <v>15</v>
+      </c>
+      <c r="C2" s="18" t="s">
+        <v>1743</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" s="18" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A3" s="18" t="s">
+        <v>16</v>
+      </c>
+      <c r="B3" s="16" t="s">
+        <v>15</v>
+      </c>
+      <c r="C3" s="18" t="s">
+        <v>1744</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" s="18" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A4" s="18" t="s">
+        <v>21</v>
+      </c>
+      <c r="B4" s="16" t="s">
+        <v>15</v>
+      </c>
+      <c r="C4" s="18" t="s">
+        <v>1745</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" s="18" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A5" s="18" t="s">
+        <v>26</v>
+      </c>
+      <c r="B5" s="16" t="s">
+        <v>15</v>
+      </c>
+      <c r="C5" s="18" t="s">
+        <v>1746</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" s="18" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A6" s="18" t="s">
+        <v>31</v>
+      </c>
+      <c r="B6" s="16" t="s">
+        <v>15</v>
+      </c>
+      <c r="C6" s="18" t="s">
+        <v>1747</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" s="18" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A7" s="18" t="s">
+        <v>138</v>
+      </c>
+      <c r="B7" s="16" t="s">
+        <v>15</v>
+      </c>
+      <c r="C7" s="18" t="s">
+        <v>1748</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" s="18" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A8" s="18" t="s">
+        <v>159</v>
+      </c>
+      <c r="B8" s="16" t="s">
+        <v>15</v>
+      </c>
+      <c r="C8" s="18" t="s">
+        <v>1749</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" s="18" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A9" s="18" t="s">
+        <v>165</v>
+      </c>
+      <c r="B9" s="16" t="s">
+        <v>15</v>
+      </c>
+      <c r="C9" s="18" t="s">
+        <v>1750</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" s="18" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A10" s="18" t="s">
+        <v>176</v>
+      </c>
+      <c r="B10" s="16" t="s">
+        <v>15</v>
+      </c>
+      <c r="C10" s="18" t="s">
+        <v>1751</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" s="18" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A11" s="18" t="s">
+        <v>183</v>
+      </c>
+      <c r="B11" s="16" t="s">
+        <v>15</v>
+      </c>
+      <c r="C11" s="18" t="s">
+        <v>1752</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" s="18" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A12" s="18" t="s">
+        <v>189</v>
+      </c>
+      <c r="B12" s="16" t="s">
+        <v>15</v>
+      </c>
+      <c r="C12" s="18" t="s">
+        <v>1753</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3" s="18" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A13" s="18" t="s">
+        <v>195</v>
+      </c>
+      <c r="B13" s="16" t="s">
+        <v>15</v>
+      </c>
+      <c r="C13" s="18" t="s">
+        <v>1754</v>
+      </c>
+    </row>
+    <row r="14" spans="1:3" s="18" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A14" s="18" t="s">
+        <v>201</v>
+      </c>
+      <c r="B14" s="16" t="s">
+        <v>15</v>
+      </c>
+      <c r="C14" s="18" t="s">
+        <v>1755</v>
+      </c>
+    </row>
+    <row r="15" spans="1:3" s="18" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A15" s="18" t="s">
+        <v>206</v>
+      </c>
+      <c r="B15" s="16" t="s">
+        <v>15</v>
+      </c>
+      <c r="C15" s="18" t="s">
+        <v>1756</v>
+      </c>
+    </row>
+    <row r="16" spans="1:3" s="18" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A16" s="18" t="s">
+        <v>211</v>
+      </c>
+      <c r="B16" s="16" t="s">
+        <v>15</v>
+      </c>
+      <c r="C16" s="18" t="s">
+        <v>1757</v>
+      </c>
+    </row>
+    <row r="17" spans="1:3" s="18" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A17" s="18" t="s">
+        <v>558</v>
+      </c>
+      <c r="B17" s="16" t="s">
+        <v>15</v>
+      </c>
+      <c r="C17" s="18" t="s">
+        <v>1758</v>
+      </c>
+    </row>
+    <row r="18" spans="1:3" s="18" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A18" s="18" t="s">
+        <v>563</v>
+      </c>
+      <c r="B18" s="16" t="s">
+        <v>15</v>
+      </c>
+      <c r="C18" s="18" t="s">
+        <v>1759</v>
+      </c>
+    </row>
+    <row r="19" spans="1:3" s="18" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A19" s="18" t="s">
+        <v>303</v>
+      </c>
+      <c r="B19" s="16" t="s">
+        <v>15</v>
+      </c>
+      <c r="C19" s="18" t="s">
+        <v>1760</v>
+      </c>
+    </row>
+    <row r="20" spans="1:3" s="18" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A20" s="18" t="s">
+        <v>309</v>
+      </c>
+      <c r="B20" s="16" t="s">
+        <v>15</v>
+      </c>
+      <c r="C20" s="18" t="s">
+        <v>1761</v>
+      </c>
+    </row>
+    <row r="21" spans="1:3" s="18" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A21" s="18" t="s">
+        <v>313</v>
+      </c>
+      <c r="B21" s="16" t="s">
+        <v>15</v>
+      </c>
+      <c r="C21" s="18" t="s">
+        <v>1762</v>
+      </c>
+    </row>
+    <row r="22" spans="1:3" s="18" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A22" s="18" t="s">
+        <v>319</v>
+      </c>
+      <c r="B22" s="16" t="s">
+        <v>15</v>
+      </c>
+      <c r="C22" s="18" t="s">
+        <v>1763</v>
+      </c>
+    </row>
+    <row r="23" spans="1:3" s="18" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A23" s="18" t="s">
+        <v>348</v>
+      </c>
+      <c r="B23" s="16" t="s">
+        <v>15</v>
+      </c>
+      <c r="C23" s="18" t="s">
+        <v>1764</v>
+      </c>
+    </row>
+    <row r="24" spans="1:3" s="18" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A24" s="18" t="s">
+        <v>354</v>
+      </c>
+      <c r="B24" s="16" t="s">
+        <v>15</v>
+      </c>
+      <c r="C24" s="18" t="s">
+        <v>1765</v>
+      </c>
+    </row>
+    <row r="25" spans="1:3" s="18" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A25" s="18" t="s">
+        <v>398</v>
+      </c>
+      <c r="B25" s="16" t="s">
+        <v>15</v>
+      </c>
+      <c r="C25" s="18" t="s">
+        <v>1766</v>
+      </c>
+    </row>
+    <row r="26" spans="1:3" s="18" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A26" s="18" t="s">
+        <v>375</v>
+      </c>
+      <c r="B26" s="16" t="s">
+        <v>15</v>
+      </c>
+      <c r="C26" s="18" t="s">
+        <v>1767</v>
+      </c>
+    </row>
+    <row r="28" spans="1:3" s="19" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A28" s="19" t="s">
+        <v>1768</v>
+      </c>
+      <c r="B28" s="19" t="s">
+        <v>41</v>
+      </c>
+      <c r="C28" s="19" t="s">
+        <v>1769</v>
       </c>
     </row>
   </sheetData>

</xml_diff>